<commit_message>
feat: implement standardized SVG icon system and scaffold comprehensive GRC platform modules
</commit_message>
<xml_diff>
--- a/grc_wisdom_api/scripts/verify/_tmp_reports/Annual_plan.xlsx
+++ b/grc_wisdom_api/scripts/verify/_tmp_reports/Annual_plan.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="60">
   <si>
     <t>Annual Audit Plan</t>
   </si>
   <si>
-    <t>Tab test plan 2033 (2033) — Active</t>
+    <t>2026 Internal Audit Plan (2026) — Approved</t>
   </si>
   <si>
     <t>Organisation</t>
@@ -38,7 +38,7 @@
     <t>Generated at</t>
   </si>
   <si>
-    <t>2026-08-16 17:58 UTC</t>
+    <t>2026-08-17 15:43 UTC</t>
   </si>
   <si>
     <t>Visibility</t>
@@ -77,28 +77,121 @@
     <t>Q1</t>
   </si>
   <si>
-    <t>Payment Operations (tab test)</t>
+    <t>Order to cash</t>
   </si>
   <si>
     <t>Process</t>
   </si>
   <si>
-    <t>5</t>
+    <t>3.45</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>Mahmoud Abdulaziz</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>Risk tier Medium (score 3.45).</t>
+  </si>
+  <si>
+    <t>Third-party and cloud management</t>
+  </si>
+  <si>
+    <t>ThirdParty</t>
+  </si>
+  <si>
+    <t>4.95</t>
   </si>
   <si>
     <t>High</t>
   </si>
   <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>InProgress</t>
-  </si>
-  <si>
-    <t>Highest scored entity.</t>
+    <t>160</t>
+  </si>
+  <si>
+    <t>Risk tier High (score 4.95). Never audited.</t>
+  </si>
+  <si>
+    <t>Procure to pay</t>
+  </si>
+  <si>
+    <t>3.85</t>
+  </si>
+  <si>
+    <t>Risk tier Medium (score 3.85).</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Personal data processing</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>Risk tier High (score 4.5). Never audited.</t>
+  </si>
+  <si>
+    <t>Treasury and cash management</t>
+  </si>
+  <si>
+    <t>3.83</t>
+  </si>
+  <si>
+    <t>Risk tier Medium (score 3.83).</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Business continuity and recovery</t>
+  </si>
+  <si>
+    <t>3.57</t>
+  </si>
+  <si>
+    <t>Risk tier Medium (score 3.57).</t>
+  </si>
+  <si>
+    <t>Identity and access management</t>
+  </si>
+  <si>
+    <t>4.35</t>
+  </si>
+  <si>
+    <t>Risk tier High (score 4.35).</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Payroll and HR operations</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t>Risk tier Medium (score 3.5).</t>
+  </si>
+  <si>
+    <t>Core banking platform</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>4.3</t>
+  </si>
+  <si>
+    <t>Risk tier High (score 4.3).</t>
   </si>
 </sst>
 </file>
@@ -602,7 +695,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -673,6 +766,238 @@
         <v>28</v>
       </c>
     </row>
+    <row r="3" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>